<commit_message>
Collapsing UXVis Items - No SUS or UEQ items
</commit_message>
<xml_diff>
--- a/Reproduce4 - Factor analysis - parallel screeplot/ItemsList.xlsx
+++ b/Reproduce4 - Factor analysis - parallel screeplot/ItemsList.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Eliane\My_codes\GitSuppMaterial\Phase 3 - Scale Validation\Reproduce4 - Factor analysis - parallel screeplot\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{860A9934-7D56-4A41-B178-1FEDD80FA3EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF090BD5-985B-43B4-B92A-25231E653966}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{FBF8989F-3BEB-4BD4-80AE-AEE8F4A6E270}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FBF8989F-3BEB-4BD4-80AE-AEE8F4A6E270}"/>
   </bookViews>
   <sheets>
-    <sheet name="ItemsList" sheetId="1" r:id="rId1"/>
-    <sheet name="factor_loadings" sheetId="2" r:id="rId2"/>
+    <sheet name="factor_loadings" sheetId="2" r:id="rId1"/>
+    <sheet name="ItemsList" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -533,162 +533,6 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A05B5693-C50D-466E-8E1D-6F01C7AE96AF}">
-  <dimension ref="A2:C14"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="32.453125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" t="s">
-        <v>3</v>
-      </c>
-      <c r="C3" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>0</v>
-      </c>
-      <c r="B4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>0</v>
-      </c>
-      <c r="B5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C5" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" t="s">
-        <v>10</v>
-      </c>
-      <c r="C6" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" t="s">
-        <v>12</v>
-      </c>
-      <c r="C7" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8" t="s">
-        <v>14</v>
-      </c>
-      <c r="C8" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>16</v>
-      </c>
-      <c r="B9" t="s">
-        <v>17</v>
-      </c>
-      <c r="C9" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
-        <v>16</v>
-      </c>
-      <c r="B10" t="s">
-        <v>19</v>
-      </c>
-      <c r="C10" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
-        <v>16</v>
-      </c>
-      <c r="B11" t="s">
-        <v>21</v>
-      </c>
-      <c r="C11" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
-        <v>16</v>
-      </c>
-      <c r="B12" t="s">
-        <v>23</v>
-      </c>
-      <c r="C12" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A13" t="s">
-        <v>16</v>
-      </c>
-      <c r="B13" t="s">
-        <v>25</v>
-      </c>
-      <c r="C13" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A14" t="s">
-        <v>16</v>
-      </c>
-      <c r="B14" t="s">
-        <v>27</v>
-      </c>
-      <c r="C14" t="s">
-        <v>28</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E59AB09-293F-4ECF-870C-8FC089495DEB}">
   <dimension ref="A1:O16"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -1339,4 +1183,160 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A05B5693-C50D-466E-8E1D-6F01C7AE96AF}">
+  <dimension ref="A2:C14"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="32.453125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11" t="s">
+        <v>21</v>
+      </c>
+      <c r="C11" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>16</v>
+      </c>
+      <c r="B12" t="s">
+        <v>23</v>
+      </c>
+      <c r="C12" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>16</v>
+      </c>
+      <c r="B13" t="s">
+        <v>25</v>
+      </c>
+      <c r="C13" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>16</v>
+      </c>
+      <c r="B14" t="s">
+        <v>27</v>
+      </c>
+      <c r="C14" t="s">
+        <v>28</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>